<commit_message>
Ajout d'une feature dans le module registre
</commit_message>
<xml_diff>
--- a/dev/Feuille de route.xlsx
+++ b/dev/Feuille de route.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexp\OneDrive\Bureau\My FrameWork &amp; Library\Framework\Torixyna\dev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexp\OneDrive\Bureau\Torixyna\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814FFD04-9BB1-44B5-B186-17AB49AB3FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393363F7-DDCC-4609-B16A-5929AE693DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Module</t>
   </si>
@@ -88,6 +88,9 @@
   </si>
   <si>
     <t>Fini pour le moment)</t>
+  </si>
+  <si>
+    <t>En cour…</t>
   </si>
 </sst>
 </file>
@@ -502,7 +505,9 @@
       <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">

</xml_diff>